<commit_message>
add supplier ,voucher validation pr required false
</commit_message>
<xml_diff>
--- a/public/uploads/vouchers/Double_claimable_Voucher.xlsx
+++ b/public/uploads/vouchers/Double_claimable_Voucher.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Financial_System\financial-app\public\uploads\vouchers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881D5BC4-C242-44F0-BA53-18F8127DF39F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8374287-9FF0-417C-85A5-D98A693B503A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5700" yWindow="1575" windowWidth="21120" windowHeight="13905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="44">
   <si>
     <t>slip#</t>
   </si>
@@ -180,9 +180,6 @@
   </si>
   <si>
     <t>12% VAT Purchase of Various medicines for Office Consumption with SI#125270</t>
-  </si>
-  <si>
-    <t>ghejensksnsisnisnsi</t>
   </si>
 </sst>
 </file>
@@ -464,7 +461,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -526,12 +523,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -565,61 +556,43 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -636,6 +609,24 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -650,6 +641,15 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1456,7 +1456,7 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="65" t="s">
+      <c r="N4" s="63" t="s">
         <v>2</v>
       </c>
       <c r="O4" s="48"/>
@@ -1491,12 +1491,12 @@
       <c r="K5" s="11"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="46" t="s">
+      <c r="N5" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="O5" s="35"/>
-      <c r="P5" s="35"/>
-      <c r="Q5" s="36"/>
+      <c r="O5" s="40"/>
+      <c r="P5" s="40"/>
+      <c r="Q5" s="37"/>
       <c r="R5" s="12"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
@@ -1536,10 +1536,10 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="66"/>
-      <c r="O6" s="44"/>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="45"/>
+      <c r="N6" s="64"/>
+      <c r="O6" s="42"/>
+      <c r="P6" s="42"/>
+      <c r="Q6" s="43"/>
       <c r="R6" s="12"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
@@ -1588,12 +1588,12 @@
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="38"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="38"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
       <c r="K8" s="1"/>
       <c r="L8" s="17" t="s">
         <v>13</v>
@@ -1615,37 +1615,37 @@
       <c r="AA8" s="1"/>
     </row>
     <row r="9" spans="1:27" ht="18" customHeight="1">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="62" t="s">
+      <c r="B9" s="40"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="50" t="s">
+      <c r="F9" s="40"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="L9" s="52" t="s">
+      <c r="L9" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="M9" s="34" t="s">
+      <c r="M9" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="35"/>
-      <c r="R9" s="35"/>
-      <c r="S9" s="35"/>
-      <c r="T9" s="35"/>
-      <c r="U9" s="36"/>
+      <c r="N9" s="40"/>
+      <c r="O9" s="40"/>
+      <c r="P9" s="40"/>
+      <c r="Q9" s="40"/>
+      <c r="R9" s="40"/>
+      <c r="S9" s="40"/>
+      <c r="T9" s="40"/>
+      <c r="U9" s="37"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
       <c r="X9" s="1"/>
@@ -1654,31 +1654,31 @@
       <c r="AA9" s="1"/>
     </row>
     <row r="10" spans="1:27" ht="18" customHeight="1">
-      <c r="A10" s="63" t="s">
+      <c r="A10" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="64" t="s">
+      <c r="B10" s="44"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="51"/>
-      <c r="L10" s="51"/>
-      <c r="M10" s="37"/>
-      <c r="N10" s="38"/>
-      <c r="O10" s="38"/>
-      <c r="P10" s="38"/>
-      <c r="Q10" s="38"/>
-      <c r="R10" s="38"/>
-      <c r="S10" s="38"/>
-      <c r="T10" s="38"/>
-      <c r="U10" s="39"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="35"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="38"/>
+      <c r="N10" s="44"/>
+      <c r="O10" s="44"/>
+      <c r="P10" s="44"/>
+      <c r="Q10" s="44"/>
+      <c r="R10" s="44"/>
+      <c r="S10" s="44"/>
+      <c r="T10" s="44"/>
+      <c r="U10" s="33"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
       <c r="X10" s="1"/>
@@ -1699,11 +1699,11 @@
       <c r="H11" s="48"/>
       <c r="I11" s="48"/>
       <c r="J11" s="49"/>
-      <c r="K11" s="41" t="s">
+      <c r="K11" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="36"/>
-      <c r="M11" s="57" t="s">
+      <c r="L11" s="37"/>
+      <c r="M11" s="61" t="s">
         <v>23</v>
       </c>
       <c r="N11" s="48"/>
@@ -1752,8 +1752,8 @@
       <c r="J12" s="18">
         <v>13</v>
       </c>
-      <c r="K12" s="37"/>
-      <c r="L12" s="39"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="33"/>
       <c r="M12" s="18">
         <v>16</v>
       </c>
@@ -1789,35 +1789,35 @@
       <c r="AA12" s="1"/>
     </row>
     <row r="13" spans="1:27" ht="24" customHeight="1">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="36"/>
-      <c r="K13" s="42" t="s">
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="L13" s="36"/>
-      <c r="M13" s="46" t="s">
+      <c r="L13" s="37"/>
+      <c r="M13" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="N13" s="36"/>
-      <c r="O13" s="69">
+      <c r="N13" s="37"/>
+      <c r="O13" s="67">
         <v>13195.09</v>
       </c>
-      <c r="P13" s="35"/>
-      <c r="Q13" s="35"/>
-      <c r="R13" s="35"/>
-      <c r="S13" s="35"/>
-      <c r="T13" s="35"/>
-      <c r="U13" s="36"/>
+      <c r="P13" s="40"/>
+      <c r="Q13" s="40"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="40"/>
+      <c r="U13" s="37"/>
       <c r="V13" s="14"/>
       <c r="W13" s="14"/>
       <c r="X13" s="14"/>
@@ -1826,27 +1826,27 @@
       <c r="AA13" s="14"/>
     </row>
     <row r="14" spans="1:27" ht="24" customHeight="1">
-      <c r="A14" s="43"/>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="37"/>
-      <c r="L14" s="39"/>
-      <c r="M14" s="37"/>
-      <c r="N14" s="39"/>
-      <c r="O14" s="37"/>
-      <c r="P14" s="38"/>
-      <c r="Q14" s="38"/>
-      <c r="R14" s="38"/>
-      <c r="S14" s="38"/>
-      <c r="T14" s="38"/>
-      <c r="U14" s="39"/>
+      <c r="A14" s="41"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="33"/>
+      <c r="M14" s="38"/>
+      <c r="N14" s="33"/>
+      <c r="O14" s="38"/>
+      <c r="P14" s="44"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="44"/>
+      <c r="S14" s="44"/>
+      <c r="T14" s="44"/>
+      <c r="U14" s="33"/>
       <c r="V14" s="14"/>
       <c r="W14" s="14"/>
       <c r="X14" s="14"/>
@@ -1855,25 +1855,25 @@
       <c r="AA14" s="14"/>
     </row>
     <row r="15" spans="1:27" ht="24" customHeight="1">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="38"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="58" t="s">
+      <c r="A15" s="38"/>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="45" t="s">
         <v>27</v>
       </c>
       <c r="L15" s="49"/>
-      <c r="M15" s="68" t="s">
+      <c r="M15" s="66" t="s">
         <v>26</v>
       </c>
       <c r="N15" s="49"/>
-      <c r="O15" s="67">
+      <c r="O15" s="65">
         <v>9125.89</v>
       </c>
       <c r="P15" s="48"/>
@@ -1900,11 +1900,11 @@
       <c r="H16" s="20"/>
       <c r="I16" s="20"/>
       <c r="J16" s="20"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="49"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="67"/>
+      <c r="K16" s="45"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="66"/>
+      <c r="N16" s="68"/>
+      <c r="O16" s="65"/>
       <c r="P16" s="48"/>
       <c r="Q16" s="48"/>
       <c r="R16" s="48"/>
@@ -1929,11 +1929,11 @@
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
       <c r="J17" s="20"/>
-      <c r="K17" s="54"/>
-      <c r="L17" s="49"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="24"/>
-      <c r="O17" s="55"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="46"/>
+      <c r="M17" s="69"/>
+      <c r="N17" s="70"/>
+      <c r="O17" s="50"/>
       <c r="P17" s="48"/>
       <c r="Q17" s="48"/>
       <c r="R17" s="48"/>
@@ -1958,11 +1958,11 @@
       <c r="H18" s="20"/>
       <c r="I18" s="20"/>
       <c r="J18" s="20"/>
-      <c r="K18" s="54"/>
-      <c r="L18" s="49"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="24"/>
-      <c r="O18" s="55"/>
+      <c r="K18" s="45"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="69"/>
+      <c r="N18" s="70"/>
+      <c r="O18" s="50"/>
       <c r="P18" s="48"/>
       <c r="Q18" s="48"/>
       <c r="R18" s="48"/>
@@ -1974,7 +1974,7 @@
       <c r="X18" s="14"/>
       <c r="Y18" s="14"/>
       <c r="Z18" s="14"/>
-      <c r="AA18" s="25"/>
+      <c r="AA18" s="23"/>
     </row>
     <row r="19" spans="1:27" ht="12.75" customHeight="1">
       <c r="A19" s="47" t="s">
@@ -1989,24 +1989,24 @@
       <c r="H19" s="48"/>
       <c r="I19" s="48"/>
       <c r="J19" s="49"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="53" t="s">
+      <c r="K19" s="24"/>
+      <c r="L19" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="M19" s="42" t="s">
+      <c r="M19" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="N19" s="36"/>
-      <c r="O19" s="56">
+      <c r="N19" s="37"/>
+      <c r="O19" s="51">
         <f>SUM(O13:U18)</f>
         <v>22320.98</v>
       </c>
-      <c r="P19" s="35"/>
-      <c r="Q19" s="35"/>
-      <c r="R19" s="35"/>
-      <c r="S19" s="35"/>
-      <c r="T19" s="35"/>
-      <c r="U19" s="36"/>
+      <c r="P19" s="40"/>
+      <c r="Q19" s="40"/>
+      <c r="R19" s="40"/>
+      <c r="S19" s="40"/>
+      <c r="T19" s="40"/>
+      <c r="U19" s="37"/>
       <c r="V19" s="1"/>
       <c r="W19" s="14"/>
       <c r="X19" s="14"/>
@@ -2027,23 +2027,23 @@
       <c r="H20" s="48"/>
       <c r="I20" s="48"/>
       <c r="J20" s="49"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="39"/>
-      <c r="M20" s="37"/>
-      <c r="N20" s="39"/>
-      <c r="O20" s="37"/>
-      <c r="P20" s="38"/>
-      <c r="Q20" s="38"/>
-      <c r="R20" s="38"/>
-      <c r="S20" s="38"/>
-      <c r="T20" s="38"/>
-      <c r="U20" s="39"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="38"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="38"/>
+      <c r="P20" s="44"/>
+      <c r="Q20" s="44"/>
+      <c r="R20" s="44"/>
+      <c r="S20" s="44"/>
+      <c r="T20" s="44"/>
+      <c r="U20" s="33"/>
       <c r="V20" s="1"/>
       <c r="W20" s="1"/>
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
-      <c r="AA20" s="28"/>
+      <c r="AA20" s="26"/>
     </row>
     <row r="21" spans="1:27" ht="12.75" customHeight="1">
       <c r="A21" s="1"/>
@@ -2101,7 +2101,7 @@
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
-      <c r="AA22" s="28"/>
+      <c r="AA22" s="26"/>
     </row>
     <row r="23" spans="1:27" ht="12.75" customHeight="1">
       <c r="A23" s="1"/>
@@ -2114,8 +2114,8 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
-      <c r="K23" s="29"/>
-      <c r="L23" s="30" t="s">
+      <c r="K23" s="27"/>
+      <c r="L23" s="28" t="s">
         <v>31</v>
       </c>
       <c r="M23" s="1"/>
@@ -2145,8 +2145,8 @@
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
-      <c r="K24" s="30"/>
-      <c r="L24" s="30" t="s">
+      <c r="K24" s="28"/>
+      <c r="L24" s="28" t="s">
         <v>32</v>
       </c>
       <c r="M24" s="1"/>
@@ -2187,7 +2187,7 @@
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
-      <c r="V25" s="31"/>
+      <c r="V25" s="29"/>
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
@@ -2255,22 +2255,22 @@
       <c r="AA27" s="1"/>
     </row>
     <row r="28" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
-      <c r="N28" s="65" t="s">
+      <c r="N28" s="63" t="s">
         <v>33</v>
       </c>
       <c r="O28" s="48"/>
@@ -2305,12 +2305,12 @@
       <c r="K29" s="11"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
-      <c r="N29" s="46" t="s">
+      <c r="N29" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="O29" s="35"/>
-      <c r="P29" s="35"/>
-      <c r="Q29" s="36"/>
+      <c r="O29" s="40"/>
+      <c r="P29" s="40"/>
+      <c r="Q29" s="37"/>
       <c r="R29" s="12"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
@@ -2350,17 +2350,17 @@
       </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
-      <c r="N30" s="66"/>
-      <c r="O30" s="44"/>
-      <c r="P30" s="44"/>
-      <c r="Q30" s="45"/>
+      <c r="N30" s="64"/>
+      <c r="O30" s="42"/>
+      <c r="P30" s="42"/>
+      <c r="Q30" s="43"/>
       <c r="R30" s="12"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
       <c r="U30" s="13"/>
       <c r="V30" s="1"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
+      <c r="W30" s="26"/>
+      <c r="X30" s="26"/>
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
       <c r="AA30" s="1"/>
@@ -2388,7 +2388,7 @@
       <c r="T31" s="3"/>
       <c r="U31" s="16"/>
       <c r="V31" s="1"/>
-      <c r="W31" s="31"/>
+      <c r="W31" s="29"/>
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
@@ -2402,12 +2402,12 @@
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="38"/>
-      <c r="J32" s="38"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44"/>
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -2421,43 +2421,43 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
-      <c r="X32" s="28"/>
+      <c r="X32" s="26"/>
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
       <c r="AA32" s="1"/>
     </row>
     <row r="33" spans="1:27" ht="18" customHeight="1">
-      <c r="A33" s="61" t="s">
+      <c r="A33" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="62" t="s">
+      <c r="B33" s="40"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="36"/>
-      <c r="K33" s="50" t="s">
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="37"/>
+      <c r="K33" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="L33" s="52" t="s">
+      <c r="L33" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="M33" s="34" t="s">
+      <c r="M33" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="N33" s="35"/>
-      <c r="O33" s="35"/>
-      <c r="P33" s="35"/>
-      <c r="Q33" s="35"/>
-      <c r="R33" s="35"/>
-      <c r="S33" s="35"/>
-      <c r="T33" s="35"/>
-      <c r="U33" s="36"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="40"/>
+      <c r="P33" s="40"/>
+      <c r="Q33" s="40"/>
+      <c r="R33" s="40"/>
+      <c r="S33" s="40"/>
+      <c r="T33" s="40"/>
+      <c r="U33" s="37"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
       <c r="X33" s="1"/>
@@ -2466,31 +2466,31 @@
       <c r="AA33" s="1"/>
     </row>
     <row r="34" spans="1:27" ht="18" customHeight="1">
-      <c r="A34" s="63" t="s">
+      <c r="A34" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="38"/>
-      <c r="C34" s="38"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="64" t="s">
+      <c r="B34" s="44"/>
+      <c r="C34" s="44"/>
+      <c r="D34" s="33"/>
+      <c r="E34" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="F34" s="38"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="38"/>
-      <c r="I34" s="38"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="51"/>
-      <c r="L34" s="51"/>
-      <c r="M34" s="37"/>
-      <c r="N34" s="38"/>
-      <c r="O34" s="38"/>
-      <c r="P34" s="38"/>
-      <c r="Q34" s="38"/>
-      <c r="R34" s="38"/>
-      <c r="S34" s="38"/>
-      <c r="T34" s="38"/>
-      <c r="U34" s="39"/>
+      <c r="F34" s="44"/>
+      <c r="G34" s="44"/>
+      <c r="H34" s="44"/>
+      <c r="I34" s="44"/>
+      <c r="J34" s="33"/>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="38"/>
+      <c r="N34" s="44"/>
+      <c r="O34" s="44"/>
+      <c r="P34" s="44"/>
+      <c r="Q34" s="44"/>
+      <c r="R34" s="44"/>
+      <c r="S34" s="44"/>
+      <c r="T34" s="44"/>
+      <c r="U34" s="33"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
@@ -2511,11 +2511,11 @@
       <c r="H35" s="48"/>
       <c r="I35" s="48"/>
       <c r="J35" s="49"/>
-      <c r="K35" s="41" t="s">
+      <c r="K35" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="L35" s="36"/>
-      <c r="M35" s="57" t="s">
+      <c r="L35" s="37"/>
+      <c r="M35" s="61" t="s">
         <v>23</v>
       </c>
       <c r="N35" s="48"/>
@@ -2564,8 +2564,8 @@
       <c r="J36" s="18">
         <v>13</v>
       </c>
-      <c r="K36" s="37"/>
-      <c r="L36" s="39"/>
+      <c r="K36" s="38"/>
+      <c r="L36" s="33"/>
       <c r="M36" s="18">
         <v>16</v>
       </c>
@@ -2601,36 +2601,36 @@
       <c r="AA36" s="1"/>
     </row>
     <row r="37" spans="1:27" ht="24" customHeight="1">
-      <c r="A37" s="42" t="s">
+      <c r="A37" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B37" s="35"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="35"/>
-      <c r="F37" s="35"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="35"/>
-      <c r="J37" s="36"/>
-      <c r="K37" s="42" t="s">
+      <c r="B37" s="40"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="40"/>
+      <c r="H37" s="40"/>
+      <c r="I37" s="40"/>
+      <c r="J37" s="37"/>
+      <c r="K37" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="L37" s="36"/>
-      <c r="M37" s="46" t="s">
+      <c r="L37" s="37"/>
+      <c r="M37" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="N37" s="36"/>
-      <c r="O37" s="40">
+      <c r="N37" s="37"/>
+      <c r="O37" s="59">
         <f>O13*0.12</f>
         <v>1583.4108000000001</v>
       </c>
-      <c r="P37" s="35"/>
-      <c r="Q37" s="35"/>
-      <c r="R37" s="35"/>
-      <c r="S37" s="35"/>
-      <c r="T37" s="35"/>
-      <c r="U37" s="36"/>
+      <c r="P37" s="40"/>
+      <c r="Q37" s="40"/>
+      <c r="R37" s="40"/>
+      <c r="S37" s="40"/>
+      <c r="T37" s="40"/>
+      <c r="U37" s="37"/>
       <c r="V37" s="14"/>
       <c r="W37" s="14"/>
       <c r="X37" s="14"/>
@@ -2639,27 +2639,27 @@
       <c r="AA37" s="14"/>
     </row>
     <row r="38" spans="1:27" ht="24" customHeight="1">
-      <c r="A38" s="43"/>
-      <c r="B38" s="44"/>
-      <c r="C38" s="44"/>
-      <c r="D38" s="44"/>
-      <c r="E38" s="44"/>
-      <c r="F38" s="44"/>
-      <c r="G38" s="44"/>
-      <c r="H38" s="44"/>
-      <c r="I38" s="44"/>
-      <c r="J38" s="45"/>
-      <c r="K38" s="37"/>
-      <c r="L38" s="39"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="39"/>
-      <c r="O38" s="37"/>
-      <c r="P38" s="38"/>
-      <c r="Q38" s="38"/>
-      <c r="R38" s="38"/>
-      <c r="S38" s="38"/>
-      <c r="T38" s="38"/>
-      <c r="U38" s="39"/>
+      <c r="A38" s="41"/>
+      <c r="B38" s="42"/>
+      <c r="C38" s="42"/>
+      <c r="D38" s="42"/>
+      <c r="E38" s="42"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="42"/>
+      <c r="I38" s="42"/>
+      <c r="J38" s="43"/>
+      <c r="K38" s="38"/>
+      <c r="L38" s="33"/>
+      <c r="M38" s="38"/>
+      <c r="N38" s="33"/>
+      <c r="O38" s="38"/>
+      <c r="P38" s="44"/>
+      <c r="Q38" s="44"/>
+      <c r="R38" s="44"/>
+      <c r="S38" s="44"/>
+      <c r="T38" s="44"/>
+      <c r="U38" s="33"/>
       <c r="V38" s="14"/>
       <c r="W38" s="14"/>
       <c r="X38" s="14"/>
@@ -2668,25 +2668,25 @@
       <c r="AA38" s="14"/>
     </row>
     <row r="39" spans="1:27" ht="24" customHeight="1">
-      <c r="A39" s="37"/>
-      <c r="B39" s="38"/>
-      <c r="C39" s="38"/>
-      <c r="D39" s="38"/>
-      <c r="E39" s="38"/>
-      <c r="F39" s="38"/>
-      <c r="G39" s="38"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="38"/>
-      <c r="J39" s="39"/>
-      <c r="K39" s="58" t="s">
+      <c r="A39" s="38"/>
+      <c r="B39" s="44"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="44"/>
+      <c r="F39" s="44"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="44"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="45" t="s">
         <v>43</v>
       </c>
       <c r="L39" s="49"/>
-      <c r="M39" s="23" t="s">
+      <c r="M39" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="N39" s="24"/>
-      <c r="O39" s="59">
+      <c r="N39" s="22"/>
+      <c r="O39" s="62">
         <f>O15*0.12</f>
         <v>1095.1068</v>
       </c>
@@ -2714,11 +2714,11 @@
       <c r="H40" s="20"/>
       <c r="I40" s="20"/>
       <c r="J40" s="20"/>
-      <c r="K40" s="54"/>
-      <c r="L40" s="49"/>
-      <c r="M40" s="23"/>
-      <c r="N40" s="24"/>
-      <c r="O40" s="55"/>
+      <c r="K40" s="45"/>
+      <c r="L40" s="46"/>
+      <c r="M40" s="69"/>
+      <c r="N40" s="70"/>
+      <c r="O40" s="50"/>
       <c r="P40" s="48"/>
       <c r="Q40" s="48"/>
       <c r="R40" s="48"/>
@@ -2743,11 +2743,11 @@
       <c r="H41" s="20"/>
       <c r="I41" s="20"/>
       <c r="J41" s="20"/>
-      <c r="K41" s="54"/>
-      <c r="L41" s="49"/>
-      <c r="M41" s="23"/>
-      <c r="N41" s="24"/>
-      <c r="O41" s="55"/>
+      <c r="K41" s="45"/>
+      <c r="L41" s="46"/>
+      <c r="M41" s="69"/>
+      <c r="N41" s="70"/>
+      <c r="O41" s="50"/>
       <c r="P41" s="48"/>
       <c r="Q41" s="48"/>
       <c r="R41" s="48"/>
@@ -2772,11 +2772,11 @@
       <c r="H42" s="20"/>
       <c r="I42" s="20"/>
       <c r="J42" s="20"/>
-      <c r="K42" s="54"/>
-      <c r="L42" s="49"/>
-      <c r="M42" s="23"/>
-      <c r="N42" s="24"/>
-      <c r="O42" s="55"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="46"/>
+      <c r="M42" s="69"/>
+      <c r="N42" s="70"/>
+      <c r="O42" s="50"/>
       <c r="P42" s="48"/>
       <c r="Q42" s="48"/>
       <c r="R42" s="48"/>
@@ -2803,25 +2803,25 @@
       <c r="H43" s="48"/>
       <c r="I43" s="48"/>
       <c r="J43" s="49"/>
-      <c r="K43" s="26"/>
-      <c r="L43" s="53" t="s">
+      <c r="K43" s="24"/>
+      <c r="L43" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="M43" s="42" t="str">
+      <c r="M43" s="39" t="str">
         <f>M37</f>
         <v>PHP</v>
       </c>
-      <c r="N43" s="36"/>
-      <c r="O43" s="56">
+      <c r="N43" s="37"/>
+      <c r="O43" s="51">
         <f>SUM(O37:U42)</f>
         <v>2678.5176000000001</v>
       </c>
-      <c r="P43" s="35"/>
-      <c r="Q43" s="35"/>
-      <c r="R43" s="35"/>
-      <c r="S43" s="35"/>
-      <c r="T43" s="35"/>
-      <c r="U43" s="36"/>
+      <c r="P43" s="40"/>
+      <c r="Q43" s="40"/>
+      <c r="R43" s="40"/>
+      <c r="S43" s="40"/>
+      <c r="T43" s="40"/>
+      <c r="U43" s="37"/>
       <c r="V43" s="1"/>
       <c r="W43" s="1"/>
       <c r="X43" s="1"/>
@@ -2842,17 +2842,17 @@
       <c r="H44" s="48"/>
       <c r="I44" s="48"/>
       <c r="J44" s="49"/>
-      <c r="K44" s="27"/>
-      <c r="L44" s="39"/>
-      <c r="M44" s="37"/>
-      <c r="N44" s="39"/>
-      <c r="O44" s="37"/>
-      <c r="P44" s="38"/>
-      <c r="Q44" s="38"/>
-      <c r="R44" s="38"/>
-      <c r="S44" s="38"/>
-      <c r="T44" s="38"/>
-      <c r="U44" s="39"/>
+      <c r="K44" s="25"/>
+      <c r="L44" s="33"/>
+      <c r="M44" s="38"/>
+      <c r="N44" s="33"/>
+      <c r="O44" s="38"/>
+      <c r="P44" s="44"/>
+      <c r="Q44" s="44"/>
+      <c r="R44" s="44"/>
+      <c r="S44" s="44"/>
+      <c r="T44" s="44"/>
+      <c r="U44" s="33"/>
       <c r="V44" s="1"/>
       <c r="W44" s="1"/>
       <c r="X44" s="1"/>
@@ -5272,9 +5272,7 @@
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
       <c r="D128" s="1"/>
-      <c r="E128" s="1" t="s">
-        <v>44</v>
-      </c>
+      <c r="E128" s="1"/>
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
       <c r="H128" s="1"/>
@@ -30587,7 +30585,7 @@
       <c r="AA1000" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="63">
+  <mergeCells count="69">
     <mergeCell ref="N4:Q4"/>
     <mergeCell ref="N5:Q5"/>
     <mergeCell ref="N6:Q6"/>
@@ -30604,12 +30602,16 @@
     <mergeCell ref="M9:U10"/>
     <mergeCell ref="O13:U14"/>
     <mergeCell ref="M13:N14"/>
-    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
     <mergeCell ref="O16:U16"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="O17:U17"/>
     <mergeCell ref="K18:L18"/>
     <mergeCell ref="O18:U18"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
     <mergeCell ref="N28:Q28"/>
     <mergeCell ref="N29:Q29"/>
     <mergeCell ref="N30:Q30"/>
@@ -30621,6 +30623,13 @@
     <mergeCell ref="E33:J33"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="E34:J34"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="M33:U34"/>
+    <mergeCell ref="O37:U38"/>
+    <mergeCell ref="M37:N38"/>
+    <mergeCell ref="M35:U35"/>
+    <mergeCell ref="O39:U39"/>
+    <mergeCell ref="M40:N40"/>
     <mergeCell ref="O41:U41"/>
     <mergeCell ref="K42:L42"/>
     <mergeCell ref="O42:U42"/>
@@ -30628,9 +30637,8 @@
     <mergeCell ref="M43:N44"/>
     <mergeCell ref="O43:U44"/>
     <mergeCell ref="A44:J44"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M41:N41"/>
+    <mergeCell ref="M42:N42"/>
     <mergeCell ref="L19:L20"/>
     <mergeCell ref="L33:L34"/>
     <mergeCell ref="L43:L44"/>
@@ -30643,14 +30651,10 @@
     <mergeCell ref="K40:L40"/>
     <mergeCell ref="A19:J19"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="M33:U34"/>
-    <mergeCell ref="O37:U38"/>
     <mergeCell ref="K35:L36"/>
     <mergeCell ref="A37:J39"/>
     <mergeCell ref="K37:L38"/>
-    <mergeCell ref="M37:N38"/>
-    <mergeCell ref="M35:U35"/>
-    <mergeCell ref="O39:U39"/>
+    <mergeCell ref="K16:L16"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.75" header="0" footer="0"/>

</xml_diff>